<commit_message>
refactor: Merge client CSS files and remove brand-kit overrides
- Merged business.css, client_dashboard.css into client.css
- Removed hardcoded colors, using CSS variables from brand-kit
- Cleaned up duplicate styles
- Improved consistency with brand design system
- Deleted business.css and client_dashboard.css

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/orders/uploads/sample.xlsx
+++ b/static/orders/uploads/sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\00-web-dev\django-ezzydelivery\ezzydelivery\orders\static\orders\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461ABAD7-59F0-4E2A-89CC-934652383C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AABC2A9-40A7-4A2F-81A6-A81EEFD01D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16530" yWindow="18660" windowWidth="21600" windowHeight="11295" xr2:uid="{9148E6BE-6549-4C07-B121-B02B966CEE9F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9148E6BE-6549-4C07-B121-B02B966CEE9F}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="1" r:id="rId1"/>
@@ -119,7 +119,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -250,6 +250,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -602,9 +610,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -963,7 +973,7 @@
   <dimension ref="A1:Y2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" customWidth="1"/>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -973,24 +983,23 @@
     <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1021,49 +1030,49 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>